<commit_message>
fix: PurchaseManager 버그 수정.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <sheetData>
     <row r="1">
@@ -1561,238 +1561,274 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>PURCHASE_NETWORK_UNAVAILABLE</t>
+          <t>PURCHASE_INTERRUPTED_SNAPSHOT_KIND_INVALID</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Network unavailable.</t>
+          <t>Interrupted purchase snapshot has invalid purchase kind.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>PURCHASE_PRODUCT_FETCH_FAILED</t>
+          <t>PURCHASE_INTERRUPTED_SNAPSHOT_PRODUCT_ID_MISSING</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Failed to fetch products from store.</t>
+          <t>Interrupted purchase snapshot is missing internalProductId.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>PURCHASE_PRODUCT_NOT_FOUND</t>
+          <t>PURCHASE_INTERRUPTED_STORAGE_UNAVAILABLE</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Product not found in TB_PRODUCT.</t>
+          <t>PurchaseStorage is not available for interrupted purchase retry.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PURCHASE_PURCHASE_IN_PROGRESS</t>
+          <t>PURCHASE_NETWORK_UNAVAILABLE</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Another purchase is already in progress.</t>
+          <t>Network unavailable.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>PURCHASE_PURCHASE_REQUEST_FAILED</t>
+          <t>PURCHASE_PRODUCT_FETCH_FAILED</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Store purchase request failed before verification.</t>
+          <t>Failed to fetch products from store.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>PURCHASE_RECENT_CALL_FAILED</t>
+          <t>PURCHASE_PRODUCT_NOT_FOUND</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Failed to fetch recent purchases.</t>
+          <t>Product not found in TB_PRODUCT.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>PURCHASE_RECENT_NOT_FOUND</t>
+          <t>PURCHASE_PURCHASE_IN_PROGRESS</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>No recent rental purchase within 30 days.</t>
+          <t>Another purchase is already in progress.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>PURCHASE_RENTAL_LATEST_CALL_FAILED</t>
+          <t>PURCHASE_PURCHASE_REQUEST_FAILED</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Failed to fetch latest rental purchase within 30 days.</t>
+          <t>Store purchase request failed before verification.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>PURCHASE_RENTAL_LATEST_NOT_FOUND</t>
+          <t>PURCHASE_RECENT_CALL_FAILED</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>No recent rental purchase within 30 days.</t>
+          <t>Failed to fetch recent purchases.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>PURCHASE_RESTORE_FAILED</t>
+          <t>PURCHASE_RECENT_NOT_FOUND</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Restore transactions failed at store.</t>
+          <t>No recent rental purchase within 30 days.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>PURCHASE_SEASON_PASS_ALREADY_OWNED</t>
+          <t>PURCHASE_RENTAL_LATEST_CALL_FAILED</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Season pass duplicate purchase is not allowed.</t>
+          <t>Failed to fetch latest rental purchase within 30 days.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>PURCHASE_STORE_FAILED</t>
+          <t>PURCHASE_RENTAL_LATEST_NOT_FOUND</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Purchase store failed</t>
+          <t>No recent rental purchase within 30 days.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>PURCHASE_STORE_NOT_SET</t>
+          <t>PURCHASE_RESTORE_FAILED</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>PurchaseStore not set. Call SetPurchaseStore().</t>
+          <t>Restore transactions failed at store.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>PURCHASE_UNAUTHENTICATED</t>
+          <t>PURCHASE_SEASON_PASS_ALREADY_OWNED</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Authentication required.</t>
+          <t>Season pass duplicate purchase is not allowed.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>PURCHASE_UNSUPPORTED_PLATFORM</t>
+          <t>PURCHASE_STORE_FAILED</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>PurchaseManager is not supported in Editor.</t>
+          <t>Purchase store failed</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>PURCHASE_VERIFY_CALL_FAILED</t>
+          <t>PURCHASE_STORE_NOT_SET</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>verifyPurchase callable failed.</t>
+          <t>PurchaseStore not set. Call SetPurchaseStore().</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>PURCHASE_VERIFY_FAILED_PRECONDITION</t>
+          <t>PURCHASE_UNAUTHENTICATED</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>verifyPurchase failed precondition.</t>
+          <t>Authentication required.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>PURCHASE_VERIFY_INVALID_ARGUMENT</t>
+          <t>PURCHASE_UNSUPPORTED_PLATFORM</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>verifyPurchase was called with invalid arguments.</t>
+          <t>PurchaseManager is not supported in Editor.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>PURCHASE_VERIFY_REJECTED_UNKNOWN</t>
+          <t>PURCHASE_VERIFY_CALL_FAILED</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>verifyPurchase rejected purchase with unknown reason.</t>
+          <t>verifyPurchase callable failed.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
+          <t>PURCHASE_VERIFY_FAILED_PRECONDITION</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>verifyPurchase failed precondition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>PURCHASE_VERIFY_INVALID_ARGUMENT</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>verifyPurchase was called with invalid arguments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>PURCHASE_VERIFY_REJECTED_UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>verifyPurchase rejected purchase with unknown reason.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
           <t>SAVEDATA_PAYLOAD_PARSE_FAILED</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t>Failed to parse save payload json</t>
         </is>

</xml_diff>

<commit_message>
fix: PurchaseManager 로직 보완.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C107"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <sheetData>
     <row r="1">
@@ -658,6 +658,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -1831,6 +1832,71 @@
       <c r="C102" t="inlineStr">
         <is>
           <t>Failed to parse save payload json</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>COMMON_INVALID_ARGUMENT</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr"/>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Invalid request arguments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>PURCHASE_ADJUSTMENTS_CALL_FAILED</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr"/>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Failed to fetch purchase adjustments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>PURCHASE_STORE_CONFIRM_ACK_CALL_FAILED</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr"/>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>ackPurchaseStoreConfirm callable failed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>PURCHASE_REFUND_APPLY_FAILED</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr"/>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Failed to apply refund adjustment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>INVENTORY_REFUND_INSUFFICIENT</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr"/>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Insufficient inventory to revoke refund rewards.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feature: Loading scene 추가. Login 로직 구현. refactor: 스킬 정리 및 리팩토링.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <sheetData>
     <row r="1">
@@ -658,1276 +658,1312 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_CHECKSUM</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Checksum mismatch</t>
+          <t>Success</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_DELETE</t>
+          <t>CLOUDSAVE_CHECKSUM</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cloud delete failed</t>
+          <t>Checksum mismatch</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_KEYIV</t>
+          <t>CLOUDSAVE_DELETE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Key/IV error</t>
+          <t>Cloud delete failed</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_LOAD</t>
+          <t>CLOUDSAVE_KEYIV</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cloud load failed</t>
+          <t>Key/IV error</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_NOCLIENT</t>
+          <t>CLOUDSAVE_LOAD</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Client not configured</t>
+          <t>Cloud load failed</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_PAYLOAD_INVALID</t>
+          <t>CLOUDSAVE_NOCLIENT</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Payload must be JSON</t>
+          <t>Client not configured</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_SAVE</t>
+          <t>CLOUDSAVE_PAYLOAD_INVALID</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Cloud save failed</t>
+          <t>Payload must be JSON</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_SIGNIN</t>
+          <t>CLOUDSAVE_SAVE</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cloud save sign-in failed</t>
+          <t>Cloud save failed</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_SLOT_EMPTY</t>
+          <t>CLOUDSAVE_SIGNIN</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Slot is empty</t>
+          <t>Cloud save sign-in failed</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_SLOT_MISSING</t>
+          <t>CLOUDSAVE_SLOT_EMPTY</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Slot not configured</t>
+          <t>Slot is empty</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>COMMON_AUTH</t>
+          <t>CLOUDSAVE_SLOT_MISSING</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Authorization error</t>
+          <t>Slot not configured</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>COMMON_NETWORK</t>
+          <t>COMMON_AUTH</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Network error</t>
+          <t>Authorization error</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>COMMON_RATE_LIMIT</t>
+          <t>COMMON_NETWORK</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Too many requests</t>
+          <t>Network error</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>COMMON_SERVER</t>
+          <t>COMMON_RATE_LIMIT</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Server error</t>
+          <t>Too many requests</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>COMMON_UNKNOWN</t>
+          <t>COMMON_SERVER</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Unknown error</t>
+          <t>Server error</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FIREBASE_APPLE_BRIDGE</t>
+          <t>COMMON_UNKNOWN</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Apple sign-in bridge is not wired</t>
+          <t>Unknown error</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FIREBASE_APPLE_SIGNIN</t>
+          <t>FIREBASE_APPLE_BRIDGE</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Apple sign-in failed</t>
+          <t>Apple sign-in bridge is not wired</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FIREBASE_APPLE_TOKEN</t>
+          <t>FIREBASE_APPLE_SIGNIN</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Apple identity token is empty</t>
+          <t>Apple sign-in failed</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FIREBASE_DEPENDENCY</t>
+          <t>FIREBASE_APPLE_TOKEN</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Firebase dependency error</t>
+          <t>Apple identity token is empty</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FIREBASE_FACEBOOK_NOT_IMPLEMENTED</t>
+          <t>FIREBASE_DEPENDENCY</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Facebook sign-in is not implemented</t>
+          <t>Firebase dependency error</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>FIREBASE_GOOGLE_REAUTH_REQUIRED</t>
+          <t>FIREBASE_FACEBOOK_NOT_IMPLEMENTED</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Google re-authentication required</t>
+          <t>Facebook sign-in is not implemented</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>FIREBASE_GOOGLE_SIGNIN</t>
+          <t>FIREBASE_GOOGLE_REAUTH_REQUIRED</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Google sign-in failed</t>
+          <t>Google re-authentication required</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>FIREBASE_GOOGLE_TOKEN</t>
+          <t>FIREBASE_GOOGLE_SIGNIN</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Google idToken is empty</t>
+          <t>Google sign-in failed</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>FIREBASE_NOT_INITIALIZED</t>
+          <t>FIREBASE_GOOGLE_TOKEN</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Firebase is not initialized</t>
+          <t>Google idToken is empty</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>FIREBASE_NO_USER</t>
+          <t>FIREBASE_NOT_INITIALIZED</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>No signed-in user</t>
+          <t>Firebase is not initialized</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>FIREBASE_REAUTH_UNKNOWN</t>
+          <t>FIREBASE_NO_USER</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Unknown re-authentication type</t>
+          <t>No signed-in user</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>FIREBASE_SIGNIN</t>
+          <t>FIREBASE_REAUTH_UNKNOWN</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Firebase sign-in failed</t>
+          <t>Unknown re-authentication type</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>FIREBASE_TOKEN</t>
+          <t>FIREBASE_SIGNIN</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Failed to get ID token</t>
+          <t>Firebase sign-in failed</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IAP_NOT_INITIALIZED</t>
+          <t>FIREBASE_TOKEN</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Store not initialized</t>
+          <t>Failed to get ID token</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>IAP_NOT_SUPPORTED</t>
+          <t>IAP_NOT_INITIALIZED</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Unity Purchasing not available</t>
+          <t>Store not initialized</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>INVENTORY_DELTAS_NULL</t>
+          <t>IAP_NOT_SUPPORTED</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>rewards array is null</t>
+          <t>Unity Purchasing not available</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>INVENTORY_DELTA_AMOUNT_NEGATIVE</t>
+          <t>INVENTORY_DELTAS_NULL</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>reward amount is negative</t>
+          <t>rewards array is null</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>INVENTORY_DELTA_ID_EMPTY</t>
+          <t>INVENTORY_DELTA_AMOUNT_NEGATIVE</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>reward id is null or empty</t>
+          <t>reward amount is negative</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>INVENTORY_DELTA_TYPE_INVALID</t>
+          <t>INVENTORY_DELTA_ID_EMPTY</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>reward type is not Item or Currency</t>
+          <t>reward id is null or empty</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>LOCALSAVE_CANCELLED</t>
+          <t>INVENTORY_DELTA_TYPE_INVALID</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Operation cancelled</t>
+          <t>reward type is not Item or Currency</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LOCALSAVE_CHECKSUM</t>
+          <t>LOCALSAVE_CANCELLED</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Checksum mismatch</t>
+          <t>Operation cancelled</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>LOCALSAVE_FILENAME_EMPTY</t>
+          <t>LOCALSAVE_CHECKSUM</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Filename is empty</t>
+          <t>Checksum mismatch</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>LOCALSAVE_FILENAME_INVALID</t>
+          <t>LOCALSAVE_FILENAME_EMPTY</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Invalid filename</t>
+          <t>Filename is empty</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>LOCALSAVE_KEYIV</t>
+          <t>LOCALSAVE_FILENAME_INVALID</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Key/IV error</t>
+          <t>Invalid filename</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LOCALSAVE_PATH_EMPTY</t>
+          <t>LOCALSAVE_KEYIV</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Root path is empty</t>
+          <t>Key/IV error</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>LOCALSAVE_READ</t>
+          <t>LOCALSAVE_PATH_EMPTY</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Read failed</t>
+          <t>Root path is empty</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LOCALSAVE_SLOT_EMPTY</t>
+          <t>LOCALSAVE_READ</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Slot is empty</t>
+          <t>Read failed</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LOCALSAVE_SLOT_MISSING</t>
+          <t>LOCALSAVE_SLOT_EMPTY</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Slot not configured</t>
+          <t>Slot is empty</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LOCALSAVE_WRITE</t>
+          <t>LOCALSAVE_SLOT_MISSING</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Write failed</t>
+          <t>Slot not configured</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LOGIN_ANONYMOUS_EXCEPTION</t>
+          <t>LOCALSAVE_WRITE</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Anonymous sign-in exception</t>
+          <t>Write failed</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>LOGIN_ANONYMOUS_FAILED</t>
+          <t>LOGIN_ANONYMOUS_EXCEPTION</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Anonymous sign-in returned no user</t>
+          <t>Anonymous sign-in exception</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>LOGIN_APPLE_EXCEPTION</t>
+          <t>LOGIN_ANONYMOUS_FAILED</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Apple sign-in exception</t>
+          <t>Anonymous sign-in returned no user</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>LOGIN_APPLE_LINK_FAILED</t>
+          <t>LOGIN_APPLE_EXCEPTION</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Failed to link Apple credential</t>
+          <t>Apple sign-in exception</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>LOGIN_APPLE_MISSING_TOKEN</t>
+          <t>LOGIN_APPLE_LINK_FAILED</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Apple IdToken and RawNonce required</t>
+          <t>Failed to link Apple credential</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LOGIN_APPLE_SIGNIN_FAILED</t>
+          <t>LOGIN_APPLE_MISSING_TOKEN</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Failed to sign in with Apple credential</t>
+          <t>Apple IdToken and RawNonce required</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LOGIN_CREDENTIAL_UNSUPPORTED</t>
+          <t>LOGIN_APPLE_SIGNIN_FAILED</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Internal credential acquisition not supported</t>
+          <t>Failed to sign in with Apple credential</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>LOGIN_FIREBASE_DEPENDENCY</t>
+          <t>LOGIN_CREDENTIAL_UNSUPPORTED</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Firebase dependency error</t>
+          <t>Internal credential acquisition not supported</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>LOGIN_GOOGLE_EXCEPTION</t>
+          <t>LOGIN_FIREBASE_DEPENDENCY</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Google sign-in exception</t>
+          <t>Firebase dependency error</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>LOGIN_GOOGLE_LINK_FAILED</t>
+          <t>LOGIN_GOOGLE_EXCEPTION</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Failed to link Google credential</t>
+          <t>Google sign-in exception</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>LOGIN_GOOGLE_MISSING_AUTH_CODE</t>
+          <t>LOGIN_GOOGLE_LINK_FAILED</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Google ServerAuthCode is required</t>
+          <t>Failed to link Google credential</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LOGIN_GOOGLE_SIGNIN_FAILED</t>
+          <t>LOGIN_GOOGLE_MISSING_AUTH_CODE</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Failed to sign in with Google credential</t>
+          <t>Google ServerAuthCode is required</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>LOGIN_GPGS_AUTH_FAILED</t>
+          <t>LOGIN_GOOGLE_SIGNIN_FAILED</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Google Play Games authentication failed</t>
+          <t>Failed to sign in with Google credential</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>LOGIN_GPGS_EXCEPTION</t>
+          <t>LOGIN_GPGS_AUTH_FAILED</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>GPGS credential exception</t>
+          <t>Google Play Games authentication failed</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>LOGIN_GPGS_NOT_FOUND</t>
+          <t>LOGIN_GPGS_EXCEPTION</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>GooglePlayGames plugin is not installed</t>
+          <t>GPGS credential exception</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>LOGIN_GPGS_NOT_INITIALIZED</t>
+          <t>LOGIN_GPGS_NOT_FOUND</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>PlayGamesPlatform.Instance is null</t>
+          <t>GooglePlayGames plugin is not installed</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>LOGIN_GPGS_NO_AUTHENTICATE</t>
+          <t>LOGIN_GPGS_NOT_INITIALIZED</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>PlayGamesPlatform.Authenticate not found</t>
+          <t>PlayGamesPlatform.Instance is null</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>LOGIN_GPGS_NO_AUTH_CODE</t>
+          <t>LOGIN_GPGS_NO_AUTHENTICATE</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Failed to obtain server auth code from GPGS</t>
+          <t>PlayGamesPlatform.Authenticate not found</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>LOGIN_GPGS_NO_SERVER_ACCESS</t>
+          <t>LOGIN_GPGS_NO_AUTH_CODE</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>PlayGamesPlatform.RequestServerSideAccess not found</t>
+          <t>Failed to obtain server auth code from GPGS</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>LOGIN_SYNC_CANCELLED</t>
+          <t>LOGIN_GPGS_NO_SERVER_ACCESS</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Sync cancelled</t>
+          <t>PlayGamesPlatform.RequestServerSideAccess not found</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>LOGIN_SYNC_LOAD_CLOUD_FAILED</t>
+          <t>LOGIN_SYNC_CANCELLED</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Sync failed while loading cloud data</t>
+          <t>Sync cancelled</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>LOGIN_SYNC_LOAD_LOCAL_FAILED</t>
+          <t>LOGIN_SYNC_LOAD_CLOUD_FAILED</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Sync failed while loading local data</t>
+          <t>Sync failed while loading cloud data</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>LOGIN_SYNC_RESOLVE_FAILED</t>
+          <t>LOGIN_SYNC_LOAD_LOCAL_FAILED</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Sync failed while resolving conflict</t>
+          <t>Sync failed while loading local data</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>LOGIN_SYNC_SAVE_CLOUD_FAILED</t>
+          <t>LOGIN_SYNC_RESOLVE_FAILED</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Sync failed while saving cloud data</t>
+          <t>Sync failed while resolving conflict</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>LOGIN_SYNC_SAVE_LOCAL_FAILED</t>
+          <t>LOGIN_SYNC_SAVE_CLOUD_FAILED</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Sync failed while saving local data</t>
+          <t>Sync failed while saving cloud data</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>LOGIN_SYNC_SLOT_LIST_FAILED</t>
+          <t>LOGIN_SYNC_SAVE_LOCAL_FAILED</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Sync failed while listing slots</t>
+          <t>Sync failed while saving local data</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>LOGIN_UNSUPPORTED</t>
+          <t>LOGIN_SYNC_SLOT_LIST_FAILED</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>LoginType not supported on this platform</t>
+          <t>Sync failed while listing slots</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>PURCHASE_ENTITLEMENTS_CALL_FAILED</t>
+          <t>LOGIN_UNSUPPORTED</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Failed to fetch entitlements snapshot.</t>
+          <t>LoginType not supported on this platform</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>PURCHASE_FUNCTION_RESPONSE_INVALID</t>
+          <t>PURCHASE_ENTITLEMENTS_CALL_FAILED</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Callable returned invalid or null response payload.</t>
+          <t>Failed to fetch entitlements snapshot.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>PURCHASE_INIT_FAILED</t>
+          <t>PURCHASE_FUNCTION_RESPONSE_INVALID</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>IAP initialization failed.</t>
+          <t>Callable returned invalid or null response payload.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>PURCHASE_INIT_REQUIRED</t>
+          <t>PURCHASE_INIT_FAILED</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>PurchaseManager not initialized. Call InitializeAsync() first.</t>
+          <t>IAP initialization failed.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>PURCHASE_INTERRUPTED_SNAPSHOT_KIND_INVALID</t>
+          <t>PURCHASE_INIT_REQUIRED</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Interrupted purchase snapshot has invalid purchase kind.</t>
+          <t>PurchaseManager not initialized. Call InitializeAsync() first.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>PURCHASE_INTERRUPTED_SNAPSHOT_PRODUCT_ID_MISSING</t>
+          <t>PURCHASE_INTERRUPTED_SNAPSHOT_KIND_INVALID</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Interrupted purchase snapshot is missing internalProductId.</t>
+          <t>Interrupted purchase snapshot has invalid purchase kind.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>PURCHASE_INTERRUPTED_STORAGE_UNAVAILABLE</t>
+          <t>PURCHASE_INTERRUPTED_SNAPSHOT_PRODUCT_ID_MISSING</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>PurchaseStorage is not available for interrupted purchase retry.</t>
+          <t>Interrupted purchase snapshot is missing internalProductId.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PURCHASE_NETWORK_UNAVAILABLE</t>
+          <t>PURCHASE_INTERRUPTED_STORAGE_UNAVAILABLE</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Network unavailable.</t>
+          <t>PurchaseStorage is not available for interrupted purchase retry.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>PURCHASE_PRODUCT_FETCH_FAILED</t>
+          <t>PURCHASE_NETWORK_UNAVAILABLE</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Failed to fetch products from store.</t>
+          <t>Network unavailable.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>PURCHASE_PRODUCT_NOT_FOUND</t>
+          <t>PURCHASE_PRODUCT_FETCH_FAILED</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Product not found in TB_PRODUCT.</t>
+          <t>Failed to fetch products from store.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>PURCHASE_PURCHASE_IN_PROGRESS</t>
+          <t>PURCHASE_PRODUCT_NOT_FOUND</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Another purchase is already in progress.</t>
+          <t>Product not found in TB_PRODUCT.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>PURCHASE_PURCHASE_REQUEST_FAILED</t>
+          <t>PURCHASE_PURCHASE_IN_PROGRESS</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Store purchase request failed before verification.</t>
+          <t>Another purchase is already in progress.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>PURCHASE_RECENT_CALL_FAILED</t>
+          <t>PURCHASE_PURCHASE_REQUEST_FAILED</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Failed to fetch recent purchases.</t>
+          <t>Store purchase request failed before verification.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>PURCHASE_RECENT_NOT_FOUND</t>
+          <t>PURCHASE_RECENT_CALL_FAILED</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>No recent rental purchase within 30 days.</t>
+          <t>Failed to fetch recent purchases.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>PURCHASE_RENTAL_LATEST_CALL_FAILED</t>
+          <t>PURCHASE_RECENT_NOT_FOUND</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Failed to fetch latest rental purchase within 30 days.</t>
+          <t>No recent rental purchase within 30 days.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>PURCHASE_RENTAL_LATEST_NOT_FOUND</t>
+          <t>PURCHASE_RENTAL_LATEST_CALL_FAILED</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>No recent rental purchase within 30 days.</t>
+          <t>Failed to fetch latest rental purchase within 30 days.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>PURCHASE_RESTORE_FAILED</t>
+          <t>PURCHASE_RENTAL_LATEST_NOT_FOUND</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Restore transactions failed at store.</t>
+          <t>No recent rental purchase within 30 days.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>PURCHASE_SEASON_PASS_ALREADY_OWNED</t>
+          <t>PURCHASE_RESTORE_FAILED</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Season pass duplicate purchase is not allowed.</t>
+          <t>Restore transactions failed at store.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>PURCHASE_STORE_FAILED</t>
+          <t>PURCHASE_SEASON_PASS_ALREADY_OWNED</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Purchase store failed</t>
+          <t>Season pass duplicate purchase is not allowed.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>PURCHASE_STORE_NOT_SET</t>
+          <t>PURCHASE_STORE_FAILED</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>PurchaseStore not set. Call SetPurchaseStore().</t>
+          <t>Purchase store failed</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>PURCHASE_UNAUTHENTICATED</t>
+          <t>PURCHASE_STORE_NOT_SET</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Authentication required.</t>
+          <t>PurchaseStore not set. Call SetPurchaseStore().</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>PURCHASE_UNSUPPORTED_PLATFORM</t>
+          <t>PURCHASE_UNAUTHENTICATED</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>PurchaseManager is not supported in Editor.</t>
+          <t>Authentication required.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>PURCHASE_VERIFY_CALL_FAILED</t>
+          <t>PURCHASE_UNSUPPORTED_PLATFORM</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>verifyPurchase callable failed.</t>
+          <t>PurchaseManager is not supported in Editor.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PURCHASE_VERIFY_FAILED_PRECONDITION</t>
+          <t>PURCHASE_VERIFY_CALL_FAILED</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>verifyPurchase failed precondition.</t>
+          <t>verifyPurchase callable failed.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>PURCHASE_VERIFY_INVALID_ARGUMENT</t>
+          <t>PURCHASE_VERIFY_FAILED_PRECONDITION</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>verifyPurchase was called with invalid arguments.</t>
+          <t>verifyPurchase failed precondition.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>PURCHASE_VERIFY_REJECTED_UNKNOWN</t>
+          <t>PURCHASE_VERIFY_INVALID_ARGUMENT</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>verifyPurchase rejected purchase with unknown reason.</t>
+          <t>verifyPurchase was called with invalid arguments.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SAVEDATA_PAYLOAD_PARSE_FAILED</t>
+          <t>PURCHASE_VERIFY_REJECTED_UNKNOWN</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Failed to parse save payload json</t>
+          <t>verifyPurchase rejected purchase with unknown reason.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>COMMON_INVALID_ARGUMENT</t>
+          <t>SAVEDATA_PAYLOAD_PARSE_FAILED</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Invalid request arguments.</t>
+          <t>Failed to parse save payload json</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>PURCHASE_ADJUSTMENTS_CALL_FAILED</t>
+          <t>COMMON_INVALID_ARGUMENT</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Failed to fetch purchase adjustments.</t>
+          <t>Invalid request arguments.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>PURCHASE_STORE_CONFIRM_ACK_CALL_FAILED</t>
+          <t>PURCHASE_ADJUSTMENTS_CALL_FAILED</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ackPurchaseStoreConfirm callable failed.</t>
+          <t>Failed to fetch purchase adjustments.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>PURCHASE_REFUND_APPLY_FAILED</t>
+          <t>PURCHASE_STORE_CONFIRM_ACK_CALL_FAILED</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Failed to apply refund adjustment.</t>
+          <t>ackPurchaseStoreConfirm callable failed.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>INVENTORY_REFUND_INSUFFICIENT</t>
+          <t>PURCHASE_REFUND_APPLY_FAILED</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Insufficient inventory to revoke refund rewards.</t>
+          <t>Failed to apply refund adjustment.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ACCOUNT_SWITCH_UNSUPPORTED</t>
+          <t>INVENTORY_REFUND_INSUFFICIENT</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Account switch is not supported for this login combination.</t>
+          <t>Insufficient inventory to revoke refund rewards.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ACCOUNT_SWITCH_GUEST_UPGRADE_FAILED</t>
+          <t>ACCOUNT_SWITCH_UNSUPPORTED</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Failed to upgrade guest account during account switch.</t>
+          <t>Account switch is not supported for this login combination.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
+          <t>ACCOUNT_SWITCH_GUEST_UPGRADE_FAILED</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Failed to upgrade guest account during account switch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
           <t>ACCOUNT_SWITCH_LOGIN_FAILED</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
+      <c r="C111" t="inlineStr">
         <is>
           <t>Failed to sign in target account during account switch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>LOCALSAVE_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Local save not found</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>CLOUDSAVE_CONNECTION_FAILED</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr"/>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Cloud connection failed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: Account, Purchase, SaveData Manager 리팩토링.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1380" yWindow="500" windowWidth="37020" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3000" yWindow="520" windowWidth="32880" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="COMPLEX_POLICY" sheetId="1" state="visible" r:id="rId1"/>
@@ -614,8 +614,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C123"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
+  <cols>
+    <col width="44.5703125" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -673,1297 +676,1416 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_CHECKSUM</t>
+          <t>ACCOUNT_SWITCH_GUEST_UPGRADE_FAILED</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Checksum mismatch</t>
+          <t>Failed to upgrade guest account during account switch.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_DELETE</t>
+          <t>ACCOUNT_SWITCH_LOGIN_FAILED</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Cloud delete failed</t>
+          <t>Failed to sign in target account during account switch.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_KEYIV</t>
+          <t>ACCOUNT_SWITCH_UNSUPPORTED</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Key/IV error</t>
+          <t>Account switch is not supported for this login combination.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_LOAD</t>
+          <t>CLOUDSAVE_CHECKSUM</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cloud load failed</t>
+          <t>Checksum mismatch</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_NOCLIENT</t>
+          <t>CLOUDSAVE_CONNECTION_FAILED</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Client not configured</t>
+          <t>Cloud connection failed</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_PAYLOAD_INVALID</t>
+          <t>CLOUDSAVE_DELETE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Payload must be JSON</t>
+          <t>Cloud delete failed</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_SAVE</t>
+          <t>CLOUDSAVE_KEYIV</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cloud save failed</t>
+          <t>Key/IV error</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_SIGNIN</t>
+          <t>CLOUDSAVE_LOAD</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cloud save sign-in failed</t>
+          <t>Cloud load failed</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_SLOT_EMPTY</t>
+          <t>CLOUDSAVE_NOCLIENT</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Slot is empty</t>
+          <t>Client not configured</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_SLOT_MISSING</t>
+          <t>CLOUDSAVE_PAYLOAD_INVALID</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Slot not configured</t>
+          <t>Payload must be JSON</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>COMMON_AUTH</t>
+          <t>CLOUDSAVE_SAVE</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Authorization error</t>
+          <t>Cloud save failed</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>COMMON_NETWORK</t>
+          <t>CLOUDSAVE_SIGNIN</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Network error</t>
+          <t>Cloud save sign-in failed</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>COMMON_RATE_LIMIT</t>
+          <t>CLOUDSAVE_SLOT_EMPTY</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Too many requests</t>
+          <t>Slot is empty</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>COMMON_SERVER</t>
+          <t>CLOUDSAVE_SLOT_MISSING</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Server error</t>
+          <t>Slot not configured</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>COMMON_UNKNOWN</t>
+          <t>COMMON_AUTH</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Unknown error</t>
+          <t>Authorization error</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FIREBASE_APPLE_BRIDGE</t>
+          <t>COMMON_INVALID_ARGUMENT</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Apple sign-in bridge is not wired</t>
+          <t>Invalid request arguments.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FIREBASE_APPLE_SIGNIN</t>
+          <t>COMMON_NETWORK</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Apple sign-in failed</t>
+          <t>Network error</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FIREBASE_APPLE_TOKEN</t>
+          <t>COMMON_RATE_LIMIT</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Apple identity token is empty</t>
+          <t>Too many requests</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FIREBASE_DEPENDENCY</t>
+          <t>COMMON_SERVER</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Firebase dependency error</t>
+          <t>Server error</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>FIREBASE_FACEBOOK_NOT_IMPLEMENTED</t>
+          <t>COMMON_UNKNOWN</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Facebook sign-in is not implemented</t>
+          <t>Unknown error</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>FIREBASE_GOOGLE_REAUTH_REQUIRED</t>
+          <t>FIREBASE_APPLE_BRIDGE</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Google re-authentication required</t>
+          <t>Apple sign-in bridge is not wired</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>FIREBASE_GOOGLE_SIGNIN</t>
+          <t>FIREBASE_APPLE_SIGNIN</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Google sign-in failed</t>
+          <t>Apple sign-in failed</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>FIREBASE_GOOGLE_TOKEN</t>
+          <t>FIREBASE_APPLE_TOKEN</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Google idToken is empty</t>
+          <t>Apple identity token is empty</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>FIREBASE_NOT_INITIALIZED</t>
+          <t>FIREBASE_DEPENDENCY</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Firebase is not initialized</t>
+          <t>Firebase dependency error</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>FIREBASE_NO_USER</t>
+          <t>FIREBASE_FACEBOOK_NOT_IMPLEMENTED</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>No signed-in user</t>
+          <t>Facebook sign-in is not implemented</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>FIREBASE_REAUTH_UNKNOWN</t>
+          <t>FIREBASE_GOOGLE_REAUTH_REQUIRED</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Unknown re-authentication type</t>
+          <t>Google re-authentication required</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>FIREBASE_SIGNIN</t>
+          <t>FIREBASE_GOOGLE_SIGNIN</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Firebase sign-in failed</t>
+          <t>Google sign-in failed</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>FIREBASE_TOKEN</t>
+          <t>FIREBASE_GOOGLE_TOKEN</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Failed to get ID token</t>
+          <t>Google idToken is empty</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>IAP_NOT_INITIALIZED</t>
+          <t>FIREBASE_NO_USER</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Store not initialized</t>
+          <t>No signed-in user</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>IAP_NOT_SUPPORTED</t>
+          <t>FIREBASE_NOT_INITIALIZED</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Unity Purchasing not available</t>
+          <t>Firebase is not initialized</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>INVENTORY_DELTAS_NULL</t>
+          <t>FIREBASE_REAUTH_UNKNOWN</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>rewards array is null</t>
+          <t>Unknown re-authentication type</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>INVENTORY_DELTA_AMOUNT_NEGATIVE</t>
+          <t>FIREBASE_SIGNIN</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>reward amount is negative</t>
+          <t>Firebase sign-in failed</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>INVENTORY_DELTA_ID_EMPTY</t>
+          <t>FIREBASE_TOKEN</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>reward id is null or empty</t>
+          <t>Failed to get ID token</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>INVENTORY_DELTA_TYPE_INVALID</t>
+          <t>IAP_NOT_INITIALIZED</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>reward type is not Item or Currency</t>
+          <t>Store not initialized</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LOCALSAVE_CANCELLED</t>
+          <t>IAP_NOT_SUPPORTED</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Operation cancelled</t>
+          <t>Unity Purchasing not available</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>LOCALSAVE_CHECKSUM</t>
+          <t>INVENTORY_DELTA_AMOUNT_NEGATIVE</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Checksum mismatch</t>
+          <t>reward amount is negative</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>LOCALSAVE_FILENAME_EMPTY</t>
+          <t>INVENTORY_DELTA_ID_EMPTY</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Filename is empty</t>
+          <t>reward id is null or empty</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>LOCALSAVE_FILENAME_INVALID</t>
+          <t>INVENTORY_DELTA_TYPE_INVALID</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Invalid filename</t>
+          <t>reward type is not Item or Currency</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LOCALSAVE_KEYIV</t>
+          <t>INVENTORY_DELTAS_NULL</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Key/IV error</t>
+          <t>rewards array is null</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>LOCALSAVE_PATH_EMPTY</t>
+          <t>INVENTORY_REFUND_INSUFFICIENT</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Root path is empty</t>
+          <t>Insufficient inventory to revoke refund rewards.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LOCALSAVE_READ</t>
+          <t>LOCALSAVE_CANCELLED</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Read failed</t>
+          <t>Operation cancelled</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LOCALSAVE_SLOT_EMPTY</t>
+          <t>LOCALSAVE_CHECKSUM</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Slot is empty</t>
+          <t>Checksum mismatch</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LOCALSAVE_SLOT_MISSING</t>
+          <t>LOCALSAVE_FILENAME_EMPTY</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Slot not configured</t>
+          <t>Filename is empty</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LOCALSAVE_WRITE</t>
+          <t>LOCALSAVE_FILENAME_INVALID</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Write failed</t>
+          <t>Invalid filename</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>LOGIN_ANONYMOUS_EXCEPTION</t>
+          <t>LOCALSAVE_KEYIV</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Anonymous sign-in exception</t>
+          <t>Key/IV error</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>LOGIN_ANONYMOUS_FAILED</t>
+          <t>LOCALSAVE_NOT_FOUND</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Anonymous sign-in returned no user</t>
+          <t>Local save not found</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>LOGIN_APPLE_EXCEPTION</t>
+          <t>LOCALSAVE_PATH_EMPTY</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Apple sign-in exception</t>
+          <t>Root path is empty</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>LOGIN_APPLE_LINK_FAILED</t>
+          <t>LOCALSAVE_READ</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Failed to link Apple credential</t>
+          <t>Read failed</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LOGIN_APPLE_MISSING_TOKEN</t>
+          <t>LOCALSAVE_SLOT_EMPTY</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Apple IdToken and RawNonce required</t>
+          <t>Slot is empty</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LOGIN_APPLE_SIGNIN_FAILED</t>
+          <t>LOCALSAVE_SLOT_MISSING</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Failed to sign in with Apple credential</t>
+          <t>Slot not configured</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>LOGIN_CREDENTIAL_UNSUPPORTED</t>
+          <t>LOCALSAVE_WRITE</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Internal credential acquisition not supported</t>
+          <t>Write failed</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>LOGIN_FIREBASE_DEPENDENCY</t>
+          <t>LOGIN_ANONYMOUS_EXCEPTION</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Firebase dependency error</t>
+          <t>Anonymous sign-in exception</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>LOGIN_GOOGLE_EXCEPTION</t>
+          <t>LOGIN_ANONYMOUS_FAILED</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Google sign-in exception</t>
+          <t>Anonymous sign-in returned no user</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>LOGIN_GOOGLE_LINK_FAILED</t>
+          <t>LOGIN_APPLE_EXCEPTION</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Failed to link Google credential</t>
+          <t>Apple sign-in exception</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LOGIN_GOOGLE_MISSING_AUTH_CODE</t>
+          <t>LOGIN_APPLE_LINK_FAILED</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Google ServerAuthCode is required</t>
+          <t>Failed to link Apple credential</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>LOGIN_GOOGLE_SIGNIN_FAILED</t>
+          <t>LOGIN_APPLE_MISSING_TOKEN</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Failed to sign in with Google credential</t>
+          <t>Apple IdToken and RawNonce required</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>LOGIN_GPGS_AUTH_FAILED</t>
+          <t>LOGIN_APPLE_SIGNIN_FAILED</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Google Play Games authentication failed</t>
+          <t>Failed to sign in with Apple credential</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>LOGIN_GPGS_EXCEPTION</t>
+          <t>LOGIN_CREDENTIAL_UNSUPPORTED</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>GPGS credential exception</t>
+          <t>Internal credential acquisition not supported</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>LOGIN_GPGS_NOT_FOUND</t>
+          <t>LOGIN_FIREBASE_DEPENDENCY</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>GooglePlayGames plugin is not installed</t>
+          <t>Firebase dependency error</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>LOGIN_GPGS_NOT_INITIALIZED</t>
+          <t>LOGIN_GOOGLE_EXCEPTION</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>PlayGamesPlatform.Instance is null</t>
+          <t>Google sign-in exception</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>LOGIN_GPGS_NO_AUTHENTICATE</t>
+          <t>LOGIN_GOOGLE_LINK_FAILED</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>PlayGamesPlatform.Authenticate not found</t>
+          <t>Failed to link Google credential</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>LOGIN_GPGS_NO_AUTH_CODE</t>
+          <t>LOGIN_GOOGLE_MISSING_AUTH_CODE</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Failed to obtain server auth code from GPGS</t>
+          <t>Google ServerAuthCode is required</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>LOGIN_GPGS_NO_SERVER_ACCESS</t>
+          <t>LOGIN_GOOGLE_SIGNIN_FAILED</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>PlayGamesPlatform.RequestServerSideAccess not found</t>
+          <t>Failed to sign in with Google credential</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>LOGIN_SYNC_CANCELLED</t>
+          <t>LOGIN_GPGS_AUTH_FAILED</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Sync cancelled</t>
+          <t>Google Play Games authentication failed</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>LOGIN_SYNC_LOAD_CLOUD_FAILED</t>
+          <t>LOGIN_GPGS_EXCEPTION</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Sync failed while loading cloud data</t>
+          <t>GPGS credential exception</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>LOGIN_SYNC_LOAD_LOCAL_FAILED</t>
+          <t>LOGIN_GPGS_NO_AUTH_CODE</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Sync failed while loading local data</t>
+          <t>Failed to obtain server auth code from GPGS</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>LOGIN_SYNC_RESOLVE_FAILED</t>
+          <t>LOGIN_GPGS_NO_AUTHENTICATE</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Sync failed while resolving conflict</t>
+          <t>PlayGamesPlatform.Authenticate not found</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>LOGIN_SYNC_SAVE_CLOUD_FAILED</t>
+          <t>LOGIN_GPGS_NO_SERVER_ACCESS</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Sync failed while saving cloud data</t>
+          <t>PlayGamesPlatform.RequestServerSideAccess not found</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>LOGIN_SYNC_SAVE_LOCAL_FAILED</t>
+          <t>LOGIN_GPGS_NOT_FOUND</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Sync failed while saving local data</t>
+          <t>GooglePlayGames plugin is not installed</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>LOGIN_SYNC_SLOT_LIST_FAILED</t>
+          <t>LOGIN_GPGS_NOT_INITIALIZED</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Sync failed while listing slots</t>
+          <t>PlayGamesPlatform.Instance is null</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>LOGIN_UNSUPPORTED</t>
+          <t>LOGIN_SYNC_CANCELLED</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>LoginType not supported on this platform</t>
+          <t>Sync cancelled</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>PURCHASE_ENTITLEMENTS_CALL_FAILED</t>
+          <t>LOGIN_SYNC_LOAD_CLOUD_FAILED</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Failed to fetch entitlements snapshot.</t>
+          <t>Sync failed while loading cloud data</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>PURCHASE_FUNCTION_RESPONSE_INVALID</t>
+          <t>LOGIN_SYNC_LOAD_LOCAL_FAILED</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Callable returned invalid or null response payload.</t>
+          <t>Sync failed while loading local data</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>PURCHASE_INIT_FAILED</t>
+          <t>LOGIN_SYNC_RESOLVE_FAILED</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>IAP initialization failed.</t>
+          <t>Sync failed while resolving conflict</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>PURCHASE_INIT_REQUIRED</t>
+          <t>LOGIN_SYNC_SAVE_CLOUD_FAILED</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>PurchaseManager not initialized. Call InitializeAsync() first.</t>
+          <t>Sync failed while saving cloud data</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>PURCHASE_INTERRUPTED_SNAPSHOT_KIND_INVALID</t>
+          <t>LOGIN_SYNC_SAVE_LOCAL_FAILED</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Interrupted purchase snapshot has invalid purchase kind.</t>
+          <t>Sync failed while saving local data</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>PURCHASE_INTERRUPTED_SNAPSHOT_PRODUCT_ID_MISSING</t>
+          <t>LOGIN_SYNC_SLOT_LIST_FAILED</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Interrupted purchase snapshot is missing internalProductId.</t>
+          <t>Sync failed while listing slots</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PURCHASE_INTERRUPTED_STORAGE_UNAVAILABLE</t>
+          <t>LOGIN_UNSUPPORTED</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>PurchaseStorage is not available for interrupted purchase retry.</t>
+          <t>LoginType not supported on this platform</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>PURCHASE_NETWORK_UNAVAILABLE</t>
+          <t>PURCHASE_ADJUSTMENTS_CALL_FAILED</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Network unavailable.</t>
+          <t>Failed to fetch purchase adjustments.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>PURCHASE_PRODUCT_FETCH_FAILED</t>
+          <t>PURCHASE_ADJUSTMENTS_INVALID_ARGUMENT</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Failed to fetch products from store.</t>
+          <t>Invalid getPurchaseAdjustments request arguments.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>PURCHASE_PRODUCT_NOT_FOUND</t>
+          <t>PURCHASE_CLIENT_GRANT_PURCHASE_ID_EMPTY</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Product not found in TB_PRODUCT.</t>
+          <t>purchaseId is required for client grant completion.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>PURCHASE_PURCHASE_IN_PROGRESS</t>
+          <t>PURCHASE_ENTITLEMENTS_CALL_FAILED</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Another purchase is already in progress.</t>
+          <t>Failed to fetch entitlements snapshot.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>PURCHASE_PURCHASE_REQUEST_FAILED</t>
+          <t>PURCHASE_FUNCTION_CALL_FAILED</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Store purchase request failed before verification.</t>
+          <t>Purchase callable failed.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>PURCHASE_RECENT_CALL_FAILED</t>
+          <t>PURCHASE_FUNCTION_RESPONSE_INVALID</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Failed to fetch recent purchases.</t>
+          <t>Callable returned invalid or null response payload.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>PURCHASE_RECENT_NOT_FOUND</t>
+          <t>PURCHASE_INIT_FAILED</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>No recent rental purchase within 30 days.</t>
+          <t>IAP initialization failed.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>PURCHASE_RENTAL_LATEST_CALL_FAILED</t>
+          <t>PURCHASE_INIT_REQUIRED</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Failed to fetch latest rental purchase within 30 days.</t>
+          <t>PurchaseManager not initialized. Call InitializeAsync() first.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>PURCHASE_RENTAL_LATEST_NOT_FOUND</t>
+          <t>PURCHASE_INTERNAL_PRODUCT_ID_EMPTY</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>No recent rental purchase within 30 days.</t>
+          <t>internalProductId is required.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>PURCHASE_RESTORE_FAILED</t>
+          <t>PURCHASE_INTERRUPTED_SNAPSHOT_KIND_INVALID</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Restore transactions failed at store.</t>
+          <t>Interrupted purchase snapshot has invalid purchase kind.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>PURCHASE_SEASON_PASS_ALREADY_OWNED</t>
+          <t>PURCHASE_INTERRUPTED_SNAPSHOT_PRODUCT_ID_MISSING</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Season pass duplicate purchase is not allowed.</t>
+          <t>Interrupted purchase snapshot is missing internalProductId.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>PURCHASE_STORE_FAILED</t>
+          <t>PURCHASE_INTERRUPTED_STORAGE_UNAVAILABLE</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Purchase store failed</t>
+          <t>PurchaseStorage is not available for interrupted purchase retry.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>PURCHASE_STORE_NOT_SET</t>
+          <t>PURCHASE_NETWORK_UNAVAILABLE</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>PurchaseStore not set. Call SetPurchaseStore().</t>
+          <t>Network unavailable.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>PURCHASE_UNAUTHENTICATED</t>
+          <t>PURCHASE_PRODUCT_FETCH_FAILED</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Authentication required.</t>
+          <t>Failed to fetch products from store.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>PURCHASE_UNSUPPORTED_PLATFORM</t>
+          <t>PURCHASE_PRODUCT_NOT_FOUND</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>PurchaseManager is not supported in Editor.</t>
+          <t>Product not found in TB_PRODUCT.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PURCHASE_VERIFY_CALL_FAILED</t>
+          <t>PURCHASE_PURCHASE_IN_PROGRESS</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>verifyPurchase callable failed.</t>
+          <t>Another purchase is already in progress.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>PURCHASE_VERIFY_FAILED_PRECONDITION</t>
+          <t>PURCHASE_PURCHASE_REQUEST_FAILED</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>verifyPurchase failed precondition.</t>
+          <t>Store purchase request failed before verification.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>PURCHASE_VERIFY_INVALID_ARGUMENT</t>
+          <t>PURCHASE_RECENT_CALL_FAILED</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>verifyPurchase was called with invalid arguments.</t>
+          <t>Failed to fetch recent purchases.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>PURCHASE_VERIFY_REJECTED_UNKNOWN</t>
+          <t>PURCHASE_RECENT_NOT_FOUND</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>verifyPurchase rejected purchase with unknown reason.</t>
+          <t>No recent rental purchase within 30 days.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SAVEDATA_PAYLOAD_PARSE_FAILED</t>
+          <t>PURCHASE_REFUND_APPLY_FAILED</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Failed to parse save payload json</t>
+          <t>Failed to apply refund adjustment.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>COMMON_INVALID_ARGUMENT</t>
+          <t>PURCHASE_RENTAL_LATEST_CALL_FAILED</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Invalid request arguments.</t>
+          <t>Failed to fetch latest rental purchase within 30 days.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>PURCHASE_ADJUSTMENTS_CALL_FAILED</t>
+          <t>PURCHASE_RENTAL_LATEST_NOT_FOUND</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Failed to fetch purchase adjustments.</t>
+          <t>No recent rental purchase within 30 days.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>PURCHASE_STORE_CONFIRM_ACK_CALL_FAILED</t>
+          <t>PURCHASE_RESTORE_FAILED</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>ackPurchaseStoreConfirm callable failed.</t>
+          <t>Restore transactions failed at store.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>PURCHASE_REFUND_APPLY_FAILED</t>
+          <t>PURCHASE_SEASON_PASS_ALREADY_OWNED</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Failed to apply refund adjustment.</t>
+          <t>Season pass duplicate purchase is not allowed.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>INVENTORY_REFUND_INSUFFICIENT</t>
+          <t>PURCHASE_STORE_CONFIRM_ACK_CALL_FAILED</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Insufficient inventory to revoke refund rewards.</t>
+          <t>ackPurchaseStoreConfirm callable failed.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ACCOUNT_SWITCH_UNSUPPORTED</t>
+          <t>PURCHASE_STORE_FAILED</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Account switch is not supported for this login combination.</t>
+          <t>Purchase store failed</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ACCOUNT_SWITCH_GUEST_UPGRADE_FAILED</t>
+          <t>PURCHASE_STORE_NOT_SET</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Failed to upgrade guest account during account switch.</t>
+          <t>PurchaseStore not set. Call SetPurchaseStore().</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ACCOUNT_SWITCH_LOGIN_FAILED</t>
+          <t>PURCHASE_UNAUTHENTICATED</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Failed to sign in target account during account switch.</t>
+          <t>Authentication required.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>LOCALSAVE_NOT_FOUND</t>
+          <t>PURCHASE_UNSUPPORTED_PLATFORM</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Local save not found</t>
+          <t>PurchaseManager is not supported in Editor.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>CLOUDSAVE_CONNECTION_FAILED</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr"/>
+          <t>PURCHASE_VERIFY_CALL_FAILED</t>
+        </is>
+      </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Cloud connection failed</t>
+          <t>verifyPurchase callable failed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>PURCHASE_VERIFY_FAILED_PRECONDITION</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>verifyPurchase failed precondition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>PURCHASE_VERIFY_INVALID_ARGUMENT</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>verifyPurchase was called with invalid arguments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>PURCHASE_VERIFY_REJECTED_UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>verifyPurchase rejected purchase with unknown reason.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>SAVEDATA_SYNC_REQUIRED</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Primary save is not initialized. Call SyncAsync first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>SAVEDATA_PAYLOAD_PARSE_FAILED</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Failed to parse save payload json</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>SAVEDATA_SYNC_CANCELLED</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>SaveData sync resolve cancelled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>SAVEDATA_SYNC_LOAD_LOCAL_FAILED</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>SaveData sync failed to load local payload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>SAVEDATA_SYNC_RESOLVE_FAILED</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>SaveData sync conflict resolution failed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>SAVEDATA_SYNC_SAVE_CLOUD_FAILED</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>SaveData sync failed to save cloud payload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>SAVEDATA_SYNC_SAVE_LOCAL_FAILED</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>SaveData sync failed to save local payload.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feature: 만기된 mission 처리 로직 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <cols>
     <col width="44.5703125" customWidth="1" min="1" max="1"/>
@@ -661,7 +661,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -2087,6 +2086,66 @@
       <c r="C123" t="inlineStr">
         <is>
           <t>SaveData sync failed to save local payload.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>MISSION_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Mission table row not found or inactive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>MISSION_RUNTIME_MISSING</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Mission runtime is missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>MISSION_RUNTIME_STALE</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Mission runtime belongs to a stale daily period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>MISSION_NOT_CLAIMABLE</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Mission is not claimable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>MISSION_ALREADY_CLAIMED</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Mission reward already claimed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feature: RecoveryManager 해킹 방어 로직 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Common/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BE04BAF-88DB-8D4E-9345-08B7302AA28B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F49A7984-47B3-2844-B037-963071F83490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40500" yWindow="-2040" windowWidth="32880" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40500" yWindow="-2360" windowWidth="32880" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COMPLEX_POLICY" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="287">
   <si>
     <t>key</t>
   </si>
@@ -880,6 +880,14 @@
   </si>
   <si>
     <t>Recovery decode error.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RECOVERY_HMAC_FAILED</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Recovery HMAC error.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1367,7 +1375,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="44.5703125" customWidth="1"/>
@@ -2406,6 +2414,14 @@
       </c>
       <c r="C130" t="s">
         <v>283</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3">
+      <c r="A131" t="s">
+        <v>285</v>
+      </c>
+      <c r="C131" t="s">
+        <v>286</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feature: Leaderboard에 season 로직 적용, CommonErrorType 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C132"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <cols>
     <col width="44.5703125" customWidth="1" min="1" max="1"/>
@@ -2195,6 +2195,102 @@
       <c r="C132" t="inlineStr">
         <is>
           <t>Product purchase is blocked near season end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>LEADERBOARD_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Active leaderboard mapping not found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>LEADERBOARD_PLATFORM_ID_MISSING</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Platform leaderboard ID mapping is missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>LEADERBOARD_MESSAGE_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>MESSAGE row for leaderboard score is missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>LEADERBOARD_MESSAGE_SAVE_TYPE_INVALID</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Leaderboard MESSAGE.saveType must be TOTAL_SUM or TOTAL_MAX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>LEADERBOARD_SEASON_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>SEASON row for leaderboard is missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>LEADERBOARD_SEASON_TIME_INVALID</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>SEASON time range is invalid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>LEADERBOARD_SERVER_TIME_UNAVAILABLE</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Server time is unavailable for leaderboard season validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>LEADERBOARD_SEASON_NOT_ACTIVE</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Leaderboard score reporting is not allowed outside active season.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: PURCHASE 테이블 이름 수정. fix: LoginManager 버그 수정.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:E140"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <cols>
     <col width="44.5703125" customWidth="1" min="1" max="1"/>
@@ -661,7 +661,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -1769,7 +1768,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>PURCHASE_PRODUCT_FETCH_FAILED</t>
+          <t>PURCHASE_FETCH_FAILED</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -1781,12 +1780,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>PURCHASE_PRODUCT_NOT_FOUND</t>
+          <t>PURCHASE_NOT_FOUND</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Product not found in TB_PRODUCT.</t>
+          <t>Product not found in TB_PURCHASE.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: enum naming 정리. fix: compile error 수정.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="40500" yWindow="-2360" windowWidth="32880" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3680" yWindow="500" windowWidth="32880" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="COMPLEX_POLICY" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ERROR_COMMON" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ERROR_SERVER" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="COMMON_ERROR" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SERVER_ERROR" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E140"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <cols>
     <col width="44.5703125" customWidth="1" min="1" max="1"/>
@@ -2306,6 +2306,9 @@
   </sheetPr>
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
+  <cols>
+    <col width="25.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>

<commit_message>
fix: Table data 오류 수정.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:J140"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <cols>
     <col width="44.5703125" customWidth="1" min="1" max="1"/>
@@ -640,7 +640,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>enum:CommonErrorType</t>
+          <t>enum:COMMON_ERROR_TYPE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -657,10 +657,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>pk, gen:CommonErrorType</t>
-        </is>
-      </c>
-    </row>
+          <t>pk, gen:COMMON_ERROR_TYPE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -2304,7 +2305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <cols>
     <col width="25.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2330,7 +2331,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>enum:ServerErrorType</t>
+          <t>enum:SERVER_ERROR_TYPE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2347,10 +2348,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>pk, gen:ServerErrorType, code</t>
-        </is>
-      </c>
-    </row>
+          <t>pk, gen:SERVER_ERROR_TYPE, code</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: data builder 버그 수정. {table_name}@{desc} refactor: ShotTable.xlsx 데이타 파일 분리.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C155"/>
+  <dimension ref="A1:C154"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <cols>
     <col width="44.5703125" customWidth="1" min="1" max="1"/>
@@ -661,6 +661,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -2301,7 +2302,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Shop productId is empty.</t>
+          <t>Shop shopId is empty.</t>
         </is>
       </c>
     </row>
@@ -2344,132 +2345,120 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>SHOP_PSEUDO_CURRENCY_PRICE_INVALID</t>
+          <t>SHOP_PURCHASE_LIMIT_DISABLED</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Shop pseudo currency price must be zero.</t>
+          <t>Shop purchase is disabled by maxCount=0.</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>SHOP_PURCHASE_LIMIT_DISABLED</t>
+          <t>SHOP_SERVER_TIME_UNAVAILABLE</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Shop purchase is disabled by maxCount=0.</t>
+          <t>Server time is unavailable for shop purchase validation.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>SHOP_PURCHASE_LIMIT_RESET_DAYS_INVALID</t>
+          <t>SHOP_PURCHASE_LIMIT_EXCEEDED</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Shop resetDays must be &gt;= 1 when purchase limit is enabled.</t>
+          <t>Shop purchase limit exceeded.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>SHOP_SERVER_TIME_UNAVAILABLE</t>
+          <t>SHOP_WALLET_UNAVAILABLE</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Server time is unavailable for shop purchase validation.</t>
+          <t>Inventory wallet is unavailable.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>SHOP_PURCHASE_LIMIT_STATE_UNAVAILABLE</t>
+          <t>SHOP_CURRENCY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Shop purchase limit state is unavailable.</t>
+          <t>Insufficient currency for shop purchase.</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>SHOP_PURCHASE_LIMIT_EXCEEDED</t>
+          <t>SHOP_ADS_NOT_AVAILABLE</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Shop purchase limit exceeded.</t>
+          <t>Shop rewarded ad is not available.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>SHOP_WALLET_UNAVAILABLE</t>
+          <t>SHOP_ADS_SHOW_FAILED</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Inventory wallet is unavailable.</t>
+          <t>Shop rewarded ad show failed.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SHOP_CURRENCY_INSUFFICIENT</t>
+          <t>SHOP_REWARD_APPLY_FAILED</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Insufficient currency for shop purchase.</t>
+          <t>Shop reward apply failed.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>SHOP_ADS_NOT_AVAILABLE</t>
+          <t>SHOP_CAN_BUY_FAILED</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Shop rewarded ad is not available.</t>
+          <t>Shop CanBuy failed.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>SHOP_ADS_SHOW_FAILED</t>
+          <t>SHOP_BUY_FAILED</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Shop rewarded ad show failed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>SHOP_REWARD_APPLY_FAILED</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>Shop reward apply failed.</t>
+          <t>Shop BuyAsync failed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feature: shop catalog chest Level/LevelUp 기능 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C154"/>
+  <dimension ref="A1:C155"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <cols>
     <col width="44.5703125" customWidth="1" min="1" max="1"/>
@@ -2459,6 +2459,18 @@
       <c r="C154" t="inlineStr">
         <is>
           <t>Shop BuyAsync failed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>SHOP_DAILY_MANUAL_REFRESH_COUNT_EXHAUSTED</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Shop daily manual refresh count exhausted.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feature: treasure system 추가. feature: Inventory Settgings 인스팩터 개선.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3680" yWindow="500" windowWidth="32880" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="COMPLEX_POLICY" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="COMMON_ERROR" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="SERVER_ERROR" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMPLEX_POLICY" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMON_ERROR" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SERVER_ERROR" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C155"/>
+  <dimension ref="A1:C161"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <cols>
     <col width="44.5703125" customWidth="1" min="1" max="1"/>
@@ -661,7 +661,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -2471,6 +2470,84 @@
       <c r="C155" t="inlineStr">
         <is>
           <t>Shop daily manual refresh count exhausted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>TREASURE_CHEST_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr"/>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Treasure chest not found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>TREASURE_GRADE_INVALID</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr"/>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Treasure grade is invalid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>TREASURE_GROUP_EMPTY</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr"/>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Treasure group is empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>TREASURE_PROGRESS_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr"/>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Treasure progress not found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>TREASURE_REWARD_APPLY_FAILED</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr"/>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Treasure reward apply failed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>TREASURE_REWARD_GROUP_EMPTY</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr"/>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Treasure reward group is empty.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feature: TREASURE_REWARD 보상 적용 시, best fit row 적용. refactor: treasure system 네이밍 정리.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C161"/>
+  <dimension ref="A1:C160"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <cols>
     <col width="44.5703125" customWidth="1" min="1" max="1"/>
@@ -2479,7 +2479,6 @@
           <t>TREASURE_CHEST_NOT_FOUND</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr"/>
       <c r="C156" t="inlineStr">
         <is>
           <t>Treasure chest not found.</t>
@@ -2492,7 +2491,6 @@
           <t>TREASURE_GRADE_INVALID</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr"/>
       <c r="C157" t="inlineStr">
         <is>
           <t>Treasure grade is invalid.</t>
@@ -2502,50 +2500,34 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>TREASURE_GROUP_EMPTY</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr"/>
+          <t>TREASURE_REWARD_EMPTY</t>
+        </is>
+      </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Treasure group is empty.</t>
+          <t>Treasure reward is empty.</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>TREASURE_PROGRESS_NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr"/>
+          <t>TREASURE_REWARD_APPLY_FAILED</t>
+        </is>
+      </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Treasure progress not found.</t>
+          <t>Treasure reward apply failed.</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>TREASURE_REWARD_APPLY_FAILED</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr"/>
+          <t>TREASURE_REWARD_GROUP_EMPTY</t>
+        </is>
+      </c>
       <c r="C160" t="inlineStr">
-        <is>
-          <t>Treasure reward apply failed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>TREASURE_REWARD_GROUP_EMPTY</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr"/>
-      <c r="C161" t="inlineStr">
         <is>
           <t>Treasure reward group is empty.</t>
         </is>

</xml_diff>

<commit_message>
feature: builder에서 foundation version number 설정 기능 추가. feature: builder에서 sample folder에 생성 코드를 자동 복사하는 기능 추가.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C160"/>
+  <dimension ref="A1:C168"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <cols>
     <col width="44.5703125" customWidth="1" min="1" max="1"/>
@@ -2530,6 +2530,102 @@
       <c r="C160" t="inlineStr">
         <is>
           <t>Treasure reward group is empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>PUSH_UNSUPPORTED_PLATFORM</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Push is not supported on this platform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>PUSH_NOT_INITIALIZED</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>PushManager not initialized. Call InitializeAsync() first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>PUSH_PERMISSION_DENIED</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Push notification permission denied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>PUSH_TOKEN_FAILED</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Failed to acquire FCM token.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>PUSH_TOPIC_SUBSCRIBE_FAILED</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Failed to subscribe to topic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>PUSH_TOPIC_UNSUBSCRIBE_FAILED</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Failed to unsubscribe from topic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>PUSH_NOTIFICATION_SCHEDULE_FAILED</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Failed to schedule local notification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>PUSH_NOTIFICATION_CANCEL_FAILED</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Failed to cancel local notification.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: achive, mission 리네이밍. enum 카테고리별 파일 분리.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C172"/>
+  <dimension ref="A1:C176"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <cols>
     <col width="44.5703125" customWidth="1" min="1" max="1"/>
@@ -2674,6 +2674,54 @@
       <c r="C172" t="inlineStr">
         <is>
           <t>Test push notification blocked in release build.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>VERSION_CHECK_NETWORK_FAILED</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Version config request failed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>VERSION_CHECK_PARSE_FAILED</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Version config JSON parse failed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>VERSION_CHECK_RESPONSE_EMPTY</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Version config response is empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>VERSION_CHECK_URL_NOT_CONFIGURED</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Version check URL is not configured for this platform.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feature: 테스트 UI 추가 및 정리. refactor: Ability factory 적용. refactor: Item table field 이름 정리.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3680" yWindow="500" windowWidth="32880" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMPLEX_POLICY" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMON_ERROR" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SERVER_ERROR" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="COMPLEX_POLICY" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="COMMON_ERROR" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SERVER_ERROR" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -614,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C176"/>
+  <dimension ref="A1:C178"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="18"/>
   <cols>
     <col width="44.5703125" customWidth="1" min="1" max="1"/>
@@ -661,6 +661,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -2722,6 +2723,30 @@
       <c r="C176" t="inlineStr">
         <is>
           <t>Version check URL is not configured for this platform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>ABILITY_ITEM_TABLE_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Ability item table row not found for the given itemId.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>ABILITY_UNIT_TABLE_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Ability unit table row not found for the given unitId.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feature: inventory 초기화 버그 수정. feature: table field 이름 그대로 source code 생성. refactor: table field 이름을 소문자 snake case 로 수정.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3680" yWindow="500" windowWidth="32880" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="COMPLEX_POLICY" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="COMMON_ERROR" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="SERVER_ERROR" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMPLEX_POLICY" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMON_ERROR" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SERVER_ERROR" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -472,17 +472,17 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>fallbackValue</t>
+          <t>fallback_value</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>minValue</t>
+          <t>min_value</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>maxValue</t>
+          <t>max_value</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: ui system 버그 수정. refactor: shop table, pk field name 수정.
</commit_message>
<xml_diff>
--- a/input/Domains/Common/CommonTable.xlsx
+++ b/input/Domains/Common/CommonTable.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3680" yWindow="500" windowWidth="32880" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMPLEX_POLICY" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMON_ERROR" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SERVER_ERROR" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="COMPLEX_POLICY" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="COMMON_ERROR" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SERVER_ERROR" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -2344,7 +2344,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>SHOP_PURCHASE_LIMIT_DISABLED</t>
+          <t>SHOP_ITEM_PURCHASE_LIMIT_DISABLED</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -2368,7 +2368,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>SHOP_PURCHASE_LIMIT_EXCEEDED</t>
+          <t>SHOP_ITEM_PURCHASE_LIMIT_EXCEEDED</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -2464,7 +2464,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>SHOP_DAILY_MANUAL_REFRESH_COUNT_EXHAUSTED</t>
+          <t>SHOP_ITEM_DAILY_MANUAL_REFRESH_COUNT_EXHAUSTED</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">

</xml_diff>